<commit_message>
Fix Marathon de Paris: chrono H 2021 (2:04:21) et 2022 (2:05:07)
- 2021: ajout ligne manquante H=2:04:21 F=2:26:11 (record course)
- 2022: correction H 2:05:00 -> 2:05:07

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E907"/>
+  <dimension ref="A1:E908"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -11128,7 +11128,7 @@
       </c>
       <c r="D426" s="3" t="inlineStr">
         <is>
-          <t>2:05:00</t>
+          <t>2:05:07</t>
         </is>
       </c>
       <c r="E426" s="3" t="inlineStr">
@@ -23159,6 +23159,31 @@
       <c r="E907" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>Schneider Electric Marathon de Paris</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>42K</t>
+        </is>
+      </c>
+      <c r="C908" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>2:04:21</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>2:26:11</t>
         </is>
       </c>
     </row>

</xml_diff>